<commit_message>
New grouping following snapshot edits.
</commit_message>
<xml_diff>
--- a/output_tables/p_gps_pts1_groupno_old.xlsx
+++ b/output_tables/p_gps_pts1_groupno_old.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/91aba14b6835b0ae/Work-current/Restoration_Storymap/2026_02_update/home_mbp/output_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{C4DB8189-CC73-4A35-AAC0-BC9B409DE3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69F262EF-44B5-4F4F-BE9D-B6F52613FC8E}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{C4DB8189-CC73-4A35-AAC0-BC9B409DE3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D997539C-A1B7-6446-9029-B63628BB51B3}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="45" windowWidth="28320" windowHeight="15315" xr2:uid="{5898ADE9-A399-4D19-B62F-88931742D621}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{5898ADE9-A399-4D19-B62F-88931742D621}"/>
   </bookViews>
   <sheets>
     <sheet name="p_gps_pts1_groupno" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -3070,46 +3083,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E6A6468-BD93-416C-A794-27A0D1F8212C}">
   <dimension ref="A1:AJ289"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="17" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="69.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.83203125" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="69.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="46.140625" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" hidden="1" customWidth="1"/>
-    <col min="11" max="12" width="13.7109375" customWidth="1"/>
-    <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="46.1640625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" hidden="1" customWidth="1"/>
+    <col min="11" max="12" width="13.6640625" customWidth="1"/>
+    <col min="13" max="13" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="7" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="17.7109375" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="17.6640625" hidden="1" customWidth="1"/>
     <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="203.5703125" customWidth="1"/>
+    <col min="20" max="20" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.5" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="29.83203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="203.5" customWidth="1"/>
     <col min="31" max="31" width="36" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="15" style="6" customWidth="1"/>
-    <col min="34" max="34" width="15.42578125" style="6" customWidth="1"/>
-    <col min="35" max="35" width="17.85546875" style="6" customWidth="1"/>
-    <col min="36" max="36" width="16.85546875" customWidth="1"/>
-    <col min="37" max="37" width="15.42578125" customWidth="1"/>
+    <col min="34" max="34" width="15.5" style="6" customWidth="1"/>
+    <col min="35" max="35" width="17.83203125" style="6" customWidth="1"/>
+    <col min="36" max="36" width="16.83203125" customWidth="1"/>
+    <col min="37" max="37" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3216,7 +3229,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3330,7 +3343,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3444,7 +3457,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3558,7 +3571,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3672,7 +3685,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3786,7 +3799,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3900,7 +3913,7 @@
         <v>AND_west_L1</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -4014,7 +4027,7 @@
         <v>AND_west_L1</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4128,7 +4141,7 @@
         <v>AND_south_L1</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4242,7 +4255,7 @@
         <v>AND_south_L1</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -4356,7 +4369,7 @@
         <v>AND_south_L2</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4470,7 +4483,7 @@
         <v>AND_south_L2</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4584,7 +4597,7 @@
         <v>AND_south_L3</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4698,7 +4711,7 @@
         <v>AND_south_L3</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -4812,7 +4825,7 @@
         <v>AND_south_L4</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -4926,7 +4939,7 @@
         <v>AND_south_L4</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -5040,7 +5053,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -5154,7 +5167,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -5268,7 +5281,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -5382,7 +5395,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -5496,7 +5509,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -5610,7 +5623,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -5724,7 +5737,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -5838,7 +5851,7 @@
         <v>BB_test_1</v>
       </c>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -5952,7 +5965,7 @@
         <v>BB_test_1</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -6066,7 +6079,7 @@
         <v>BB_test_1</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -6180,7 +6193,7 @@
         <v>BB_test_1</v>
       </c>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -6294,7 +6307,7 @@
         <v>BB_test_1</v>
       </c>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -6408,7 +6421,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -6522,7 +6535,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -6636,7 +6649,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -6750,7 +6763,7 @@
         <v>COM_L1</v>
       </c>
     </row>
-    <row r="33" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -6864,7 +6877,7 @@
         <v>COM_L1</v>
       </c>
     </row>
-    <row r="34" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -6978,7 +6991,7 @@
         <v>COM_L2</v>
       </c>
     </row>
-    <row r="35" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -7092,7 +7105,7 @@
         <v>COM_L2</v>
       </c>
     </row>
-    <row r="36" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -7206,7 +7219,7 @@
         <v>DEL_1</v>
       </c>
     </row>
-    <row r="37" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -7320,7 +7333,7 @@
         <v>DEL_L1</v>
       </c>
     </row>
-    <row r="38" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -7434,7 +7447,7 @@
         <v>DEL_L1</v>
       </c>
     </row>
-    <row r="39" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -7548,7 +7561,7 @@
         <v>DEL_P1</v>
       </c>
     </row>
-    <row r="40" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -7662,7 +7675,7 @@
         <v>DEL_P1</v>
       </c>
     </row>
-    <row r="41" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -7776,7 +7789,7 @@
         <v>DEL_P1</v>
       </c>
     </row>
-    <row r="42" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -7890,7 +7903,7 @@
         <v>DEL_P1</v>
       </c>
     </row>
-    <row r="43" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -8004,7 +8017,7 @@
         <v>DEL_3</v>
       </c>
     </row>
-    <row r="44" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -8118,7 +8131,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -8232,7 +8245,7 @@
         <v>DEL_1</v>
       </c>
     </row>
-    <row r="46" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -8346,7 +8359,7 @@
         <v>DEL_3</v>
       </c>
     </row>
-    <row r="47" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -8460,7 +8473,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -8574,7 +8587,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -8688,7 +8701,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -8802,7 +8815,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -8916,7 +8929,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -9030,7 +9043,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -9144,7 +9157,7 @@
         <v>DB_test_2</v>
       </c>
     </row>
-    <row r="54" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -9258,7 +9271,7 @@
         <v>DB_test_2</v>
       </c>
     </row>
-    <row r="55" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -9372,7 +9385,7 @@
         <v>DB_test_2</v>
       </c>
     </row>
-    <row r="56" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -9486,7 +9499,7 @@
         <v>DB_test_2</v>
       </c>
     </row>
-    <row r="57" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -9600,7 +9613,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -9714,7 +9727,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -9828,7 +9841,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -9942,7 +9955,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -10056,7 +10069,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -10170,7 +10183,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -10284,7 +10297,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -10398,7 +10411,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -10512,7 +10525,7 @@
         <v>FDG_L1</v>
       </c>
     </row>
-    <row r="66" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -10626,7 +10639,7 @@
         <v>FDG_L1</v>
       </c>
     </row>
-    <row r="67" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -10740,7 +10753,7 @@
         <v>FDG_L2</v>
       </c>
     </row>
-    <row r="68" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -10854,7 +10867,7 @@
         <v>FDG_L2</v>
       </c>
     </row>
-    <row r="69" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -10968,7 +10981,7 @@
         <v>FDG_L1</v>
       </c>
     </row>
-    <row r="70" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -11082,7 +11095,7 @@
         <v>FDG_L1</v>
       </c>
     </row>
-    <row r="71" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -11196,7 +11209,7 @@
         <v>FDG_L2</v>
       </c>
     </row>
-    <row r="72" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -11310,7 +11323,7 @@
         <v>FDG_L2</v>
       </c>
     </row>
-    <row r="73" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -11424,7 +11437,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -11538,7 +11551,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -11652,7 +11665,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -11766,7 +11779,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -11880,7 +11893,7 @@
         <v>HAR_4</v>
       </c>
     </row>
-    <row r="78" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -11994,7 +12007,7 @@
         <v>HAR_4</v>
       </c>
     </row>
-    <row r="79" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -12108,7 +12121,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -12222,7 +12235,7 @@
         <v>HAR_deep_L1</v>
       </c>
     </row>
-    <row r="81" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -12336,7 +12349,7 @@
         <v>HAR_deep_L1</v>
       </c>
     </row>
-    <row r="82" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -12450,7 +12463,7 @@
         <v>HAR_shallow_L1</v>
       </c>
     </row>
-    <row r="83" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -12564,7 +12577,7 @@
         <v>HAR_shallow_L1</v>
       </c>
     </row>
-    <row r="84" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -12678,7 +12691,7 @@
         <v>HAR_shallow_L2</v>
       </c>
     </row>
-    <row r="85" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -12792,7 +12805,7 @@
         <v>HAR_shallow_L2</v>
       </c>
     </row>
-    <row r="86" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -12906,7 +12919,7 @@
         <v>HAR_shallow_L3</v>
       </c>
     </row>
-    <row r="87" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -13020,7 +13033,7 @@
         <v>HAR_shallow_L3</v>
       </c>
     </row>
-    <row r="88" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -13134,7 +13147,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -13248,7 +13261,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -13362,7 +13375,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -13476,7 +13489,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -13590,7 +13603,7 @@
         <v>HPT_north_2</v>
       </c>
     </row>
-    <row r="93" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -13704,7 +13717,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -13818,7 +13831,7 @@
         <v>HPT_north_2</v>
       </c>
     </row>
-    <row r="95" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -13932,7 +13945,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -14046,7 +14059,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -14160,7 +14173,7 @@
         <v>JSP_mid_south_P1</v>
       </c>
     </row>
-    <row r="98" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -14274,7 +14287,7 @@
         <v>JSP_mid_south_P1</v>
       </c>
     </row>
-    <row r="99" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -14388,7 +14401,7 @@
         <v>JSP_mid_south_P1</v>
       </c>
     </row>
-    <row r="100" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -14502,7 +14515,7 @@
         <v>JSP_mid_south_P1</v>
       </c>
     </row>
-    <row r="101" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -14616,7 +14629,7 @@
         <v>JSP_mid_north_P1</v>
       </c>
     </row>
-    <row r="102" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -14730,7 +14743,7 @@
         <v>JSP_mid_north_P1</v>
       </c>
     </row>
-    <row r="103" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -14844,7 +14857,7 @@
         <v>JSP_mid_north_P1</v>
       </c>
     </row>
-    <row r="104" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -14958,7 +14971,7 @@
         <v>JSP_mid_north_P1</v>
       </c>
     </row>
-    <row r="105" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -15072,7 +15085,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>105</v>
       </c>
@@ -15186,7 +15199,7 @@
         <v>JSP_north</v>
       </c>
     </row>
-    <row r="107" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -15300,7 +15313,7 @@
         <v>JSP_north</v>
       </c>
     </row>
-    <row r="108" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -15414,7 +15427,7 @@
         <v>JSP_south_P1</v>
       </c>
     </row>
-    <row r="109" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -15528,7 +15541,7 @@
         <v>JSP_south_P1</v>
       </c>
     </row>
-    <row r="110" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -15642,7 +15655,7 @@
         <v>JSP_south_P1</v>
       </c>
     </row>
-    <row r="111" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -15756,7 +15769,7 @@
         <v>JSP_south_P1</v>
       </c>
     </row>
-    <row r="112" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -15870,7 +15883,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>112</v>
       </c>
@@ -15984,7 +15997,7 @@
         <v>JSP_north_L1</v>
       </c>
     </row>
-    <row r="114" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -16098,7 +16111,7 @@
         <v>JSP_north_L1</v>
       </c>
     </row>
-    <row r="115" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -16212,7 +16225,7 @@
         <v>JSP_north_L2</v>
       </c>
     </row>
-    <row r="116" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -16326,7 +16339,7 @@
         <v>JSP_north_L2</v>
       </c>
     </row>
-    <row r="117" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>116</v>
       </c>
@@ -16440,7 +16453,7 @@
         <v>JSP_south_P2</v>
       </c>
     </row>
-    <row r="118" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>117</v>
       </c>
@@ -16554,7 +16567,7 @@
         <v>JSP_south_P2</v>
       </c>
     </row>
-    <row r="119" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>118</v>
       </c>
@@ -16668,7 +16681,7 @@
         <v>JSP_south_P2</v>
       </c>
     </row>
-    <row r="120" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>119</v>
       </c>
@@ -16782,7 +16795,7 @@
         <v>JSP_south_P2</v>
       </c>
     </row>
-    <row r="121" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>120</v>
       </c>
@@ -16896,7 +16909,7 @@
         <v>JSP_south_P3</v>
       </c>
     </row>
-    <row r="122" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>121</v>
       </c>
@@ -17010,7 +17023,7 @@
         <v>JSP_south_P3</v>
       </c>
     </row>
-    <row r="123" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>122</v>
       </c>
@@ -17124,7 +17137,7 @@
         <v>JSP_south_P3</v>
       </c>
     </row>
-    <row r="124" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>123</v>
       </c>
@@ -17238,7 +17251,7 @@
         <v>JSP_south_P3</v>
       </c>
     </row>
-    <row r="125" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>124</v>
       </c>
@@ -17352,7 +17365,7 @@
         <v>JSP_south_P4</v>
       </c>
     </row>
-    <row r="126" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>125</v>
       </c>
@@ -17466,7 +17479,7 @@
         <v>JSP_south_P4</v>
       </c>
     </row>
-    <row r="127" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>126</v>
       </c>
@@ -17580,7 +17593,7 @@
         <v>JSP_south_P4</v>
       </c>
     </row>
-    <row r="128" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>127</v>
       </c>
@@ -17694,7 +17707,7 @@
         <v>JSP_south_P4</v>
       </c>
     </row>
-    <row r="129" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>128</v>
       </c>
@@ -17808,7 +17821,7 @@
         <v>JSP_mid_AG1</v>
       </c>
     </row>
-    <row r="130" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>129</v>
       </c>
@@ -17922,7 +17935,7 @@
         <v>JSP_mid_BG1</v>
       </c>
     </row>
-    <row r="131" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>130</v>
       </c>
@@ -18036,7 +18049,7 @@
         <v>JSP_mid_C1</v>
       </c>
     </row>
-    <row r="132" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>131</v>
       </c>
@@ -18150,7 +18163,7 @@
         <v>JSP_mid_AG2</v>
       </c>
     </row>
-    <row r="133" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>132</v>
       </c>
@@ -18264,7 +18277,7 @@
         <v>JSP_mid_C2</v>
       </c>
     </row>
-    <row r="134" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>133</v>
       </c>
@@ -18378,7 +18391,7 @@
         <v>JSP_mid_BG2</v>
       </c>
     </row>
-    <row r="135" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>134</v>
       </c>
@@ -18492,7 +18505,7 @@
         <v>JSP_mid_C3</v>
       </c>
     </row>
-    <row r="136" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>135</v>
       </c>
@@ -18606,7 +18619,7 @@
         <v>JSP_mid_BG3</v>
       </c>
     </row>
-    <row r="137" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>136</v>
       </c>
@@ -18720,7 +18733,7 @@
         <v>JSP_mid_C4</v>
       </c>
     </row>
-    <row r="138" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>137</v>
       </c>
@@ -18834,7 +18847,7 @@
         <v>JSP_mid_BG4</v>
       </c>
     </row>
-    <row r="139" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>138</v>
       </c>
@@ -18948,7 +18961,7 @@
         <v>JSP_mid_AG3</v>
       </c>
     </row>
-    <row r="140" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>139</v>
       </c>
@@ -19062,7 +19075,7 @@
         <v>JSP_mid_AG4</v>
       </c>
     </row>
-    <row r="141" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>140</v>
       </c>
@@ -19176,7 +19189,7 @@
         <v>JSP_north_P1</v>
       </c>
     </row>
-    <row r="142" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>141</v>
       </c>
@@ -19290,7 +19303,7 @@
         <v>JSP_north_P1</v>
       </c>
     </row>
-    <row r="143" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>142</v>
       </c>
@@ -19404,7 +19417,7 @@
         <v>JSP_north_P1</v>
       </c>
     </row>
-    <row r="144" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>143</v>
       </c>
@@ -19518,7 +19531,7 @@
         <v>JSP_north_P1</v>
       </c>
     </row>
-    <row r="145" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>144</v>
       </c>
@@ -19632,7 +19645,7 @@
         <v>JSP_mid_P1</v>
       </c>
     </row>
-    <row r="146" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>145</v>
       </c>
@@ -19746,7 +19759,7 @@
         <v>JSP_mid_P1</v>
       </c>
     </row>
-    <row r="147" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>146</v>
       </c>
@@ -19860,7 +19873,7 @@
         <v>JSP_mid_P1</v>
       </c>
     </row>
-    <row r="148" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>147</v>
       </c>
@@ -19974,7 +19987,7 @@
         <v>JSP_mid_P1</v>
       </c>
     </row>
-    <row r="149" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>148</v>
       </c>
@@ -20088,7 +20101,7 @@
         <v>JSP_south_P5</v>
       </c>
     </row>
-    <row r="150" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>149</v>
       </c>
@@ -20202,7 +20215,7 @@
         <v>JSP_south_P5</v>
       </c>
     </row>
-    <row r="151" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>150</v>
       </c>
@@ -20316,7 +20329,7 @@
         <v>JSP_south_P5</v>
       </c>
     </row>
-    <row r="152" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>151</v>
       </c>
@@ -20430,7 +20443,7 @@
         <v>JSP_south_P5</v>
       </c>
     </row>
-    <row r="153" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>152</v>
       </c>
@@ -20544,7 +20557,7 @@
         <v>JSP_mid_south_2</v>
       </c>
     </row>
-    <row r="154" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>153</v>
       </c>
@@ -20658,7 +20671,7 @@
         <v>JSP_mid_south_2</v>
       </c>
     </row>
-    <row r="155" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>154</v>
       </c>
@@ -20772,7 +20785,7 @@
         <v>JSP_mid_south_2</v>
       </c>
     </row>
-    <row r="156" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>155</v>
       </c>
@@ -20886,7 +20899,7 @@
         <v>JSP_mid_south_2</v>
       </c>
     </row>
-    <row r="157" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>156</v>
       </c>
@@ -21000,7 +21013,7 @@
         <v>JSP_mid_AG1</v>
       </c>
     </row>
-    <row r="158" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>157</v>
       </c>
@@ -21114,7 +21127,7 @@
         <v>JSP_mid_BG1</v>
       </c>
     </row>
-    <row r="159" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>158</v>
       </c>
@@ -21228,7 +21241,7 @@
         <v>JSP_mid_C1</v>
       </c>
     </row>
-    <row r="160" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>159</v>
       </c>
@@ -21342,7 +21355,7 @@
         <v>JSP_mid_AG2</v>
       </c>
     </row>
-    <row r="161" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>160</v>
       </c>
@@ -21456,7 +21469,7 @@
         <v>JSP_mid_C2</v>
       </c>
     </row>
-    <row r="162" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>161</v>
       </c>
@@ -21570,7 +21583,7 @@
         <v>JSP_mid_BG2</v>
       </c>
     </row>
-    <row r="163" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>162</v>
       </c>
@@ -21684,7 +21697,7 @@
         <v>JSP_mid_C3</v>
       </c>
     </row>
-    <row r="164" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>163</v>
       </c>
@@ -21798,7 +21811,7 @@
         <v>JSP_mid_BG3</v>
       </c>
     </row>
-    <row r="165" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>164</v>
       </c>
@@ -21912,7 +21925,7 @@
         <v>JSP_mid_C4</v>
       </c>
     </row>
-    <row r="166" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>165</v>
       </c>
@@ -22026,7 +22039,7 @@
         <v>JSP_mid_BG4</v>
       </c>
     </row>
-    <row r="167" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>166</v>
       </c>
@@ -22140,7 +22153,7 @@
         <v>JSP_mid_AG3</v>
       </c>
     </row>
-    <row r="168" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>167</v>
       </c>
@@ -22254,7 +22267,7 @@
         <v>JSP_mid_AG4</v>
       </c>
     </row>
-    <row r="169" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>168</v>
       </c>
@@ -22368,7 +22381,7 @@
         <v>JSP_mid_south_2</v>
       </c>
     </row>
-    <row r="170" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>169</v>
       </c>
@@ -22482,7 +22495,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>170</v>
       </c>
@@ -22596,7 +22609,7 @@
         <v>JSP_mid_1</v>
       </c>
     </row>
-    <row r="172" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>171</v>
       </c>
@@ -22710,7 +22723,7 @@
         <v>JSP_mid_1</v>
       </c>
     </row>
-    <row r="173" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>172</v>
       </c>
@@ -22824,7 +22837,7 @@
         <v>JSP_mid_2</v>
       </c>
     </row>
-    <row r="174" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>173</v>
       </c>
@@ -22938,7 +22951,7 @@
         <v>JSP_mid_2</v>
       </c>
     </row>
-    <row r="175" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>174</v>
       </c>
@@ -23052,7 +23065,7 @@
         <v>JSP_mid_3</v>
       </c>
     </row>
-    <row r="176" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>175</v>
       </c>
@@ -23166,7 +23179,7 @@
         <v>JSP_mid_3</v>
       </c>
     </row>
-    <row r="177" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>176</v>
       </c>
@@ -23280,7 +23293,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>177</v>
       </c>
@@ -23394,7 +23407,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>178</v>
       </c>
@@ -23508,7 +23521,7 @@
         <v/>
       </c>
     </row>
-    <row r="180" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>179</v>
       </c>
@@ -23622,7 +23635,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>180</v>
       </c>
@@ -23736,7 +23749,7 @@
         <v/>
       </c>
     </row>
-    <row r="182" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>181</v>
       </c>
@@ -23850,7 +23863,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>182</v>
       </c>
@@ -23964,7 +23977,7 @@
         <v/>
       </c>
     </row>
-    <row r="184" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>183</v>
       </c>
@@ -24078,7 +24091,7 @@
         <v/>
       </c>
     </row>
-    <row r="185" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185">
         <v>184</v>
       </c>
@@ -24192,7 +24205,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>185</v>
       </c>
@@ -24306,7 +24319,7 @@
         <v>MCD_south_L1</v>
       </c>
     </row>
-    <row r="187" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>186</v>
       </c>
@@ -24420,7 +24433,7 @@
         <v>MCD_south_L1</v>
       </c>
     </row>
-    <row r="188" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>187</v>
       </c>
@@ -24534,7 +24547,7 @@
         <v>MCD_north_L1</v>
       </c>
     </row>
-    <row r="189" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189">
         <v>188</v>
       </c>
@@ -24648,7 +24661,7 @@
         <v>MCD_north_L1</v>
       </c>
     </row>
-    <row r="190" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190">
         <v>189</v>
       </c>
@@ -24762,7 +24775,7 @@
         <v/>
       </c>
     </row>
-    <row r="191" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191">
         <v>190</v>
       </c>
@@ -24876,7 +24889,7 @@
         <v/>
       </c>
     </row>
-    <row r="192" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>191</v>
       </c>
@@ -24990,7 +25003,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193">
         <v>192</v>
       </c>
@@ -25104,7 +25117,7 @@
         <v/>
       </c>
     </row>
-    <row r="194" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194">
         <v>193</v>
       </c>
@@ -25218,7 +25231,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195">
         <v>194</v>
       </c>
@@ -25332,7 +25345,7 @@
         <v/>
       </c>
     </row>
-    <row r="196" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196">
         <v>195</v>
       </c>
@@ -25446,7 +25459,7 @@
         <v>MCN_still_2</v>
       </c>
     </row>
-    <row r="197" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197">
         <v>196</v>
       </c>
@@ -25560,7 +25573,7 @@
         <v>MCN_still_2</v>
       </c>
     </row>
-    <row r="198" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>197</v>
       </c>
@@ -25674,7 +25687,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199">
         <v>198</v>
       </c>
@@ -25788,7 +25801,7 @@
         <v/>
       </c>
     </row>
-    <row r="200" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200">
         <v>199</v>
       </c>
@@ -25902,7 +25915,7 @@
         <v>MCN_south_L2</v>
       </c>
     </row>
-    <row r="201" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201">
         <v>200</v>
       </c>
@@ -26016,7 +26029,7 @@
         <v>MCN_south_L2</v>
       </c>
     </row>
-    <row r="202" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A202">
         <v>201</v>
       </c>
@@ -26130,7 +26143,7 @@
         <v>MCN_south_L1</v>
       </c>
     </row>
-    <row r="203" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A203">
         <v>202</v>
       </c>
@@ -26244,7 +26257,7 @@
         <v>MCN_south_L1</v>
       </c>
     </row>
-    <row r="204" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A204">
         <v>203</v>
       </c>
@@ -26358,7 +26371,7 @@
         <v>MCN_south_L3</v>
       </c>
     </row>
-    <row r="205" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205">
         <v>204</v>
       </c>
@@ -26472,7 +26485,7 @@
         <v>MCN_south_L3</v>
       </c>
     </row>
-    <row r="206" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206">
         <v>205</v>
       </c>
@@ -26586,7 +26599,7 @@
         <v/>
       </c>
     </row>
-    <row r="207" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207">
         <v>206</v>
       </c>
@@ -26700,7 +26713,7 @@
         <v/>
       </c>
     </row>
-    <row r="208" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208">
         <v>207</v>
       </c>
@@ -26814,7 +26827,7 @@
         <v>MRE_1</v>
       </c>
     </row>
-    <row r="209" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209">
         <v>208</v>
       </c>
@@ -26928,7 +26941,7 @@
         <v>MRE_1</v>
       </c>
     </row>
-    <row r="210" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210">
         <v>209</v>
       </c>
@@ -27042,7 +27055,7 @@
         <v>MRE_2</v>
       </c>
     </row>
-    <row r="211" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A211">
         <v>210</v>
       </c>
@@ -27156,7 +27169,7 @@
         <v>MRE_2</v>
       </c>
     </row>
-    <row r="212" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212">
         <v>211</v>
       </c>
@@ -27270,7 +27283,7 @@
         <v/>
       </c>
     </row>
-    <row r="213" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213">
         <v>212</v>
       </c>
@@ -27384,7 +27397,7 @@
         <v/>
       </c>
     </row>
-    <row r="214" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214">
         <v>213</v>
       </c>
@@ -27498,7 +27511,7 @@
         <v/>
       </c>
     </row>
-    <row r="215" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215">
         <v>214</v>
       </c>
@@ -27612,7 +27625,7 @@
         <v/>
       </c>
     </row>
-    <row r="216" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216">
         <v>215</v>
       </c>
@@ -27726,7 +27739,7 @@
         <v/>
       </c>
     </row>
-    <row r="217" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217">
         <v>216</v>
       </c>
@@ -27840,7 +27853,7 @@
         <v/>
       </c>
     </row>
-    <row r="218" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218">
         <v>217</v>
       </c>
@@ -27954,7 +27967,7 @@
         <v/>
       </c>
     </row>
-    <row r="219" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219">
         <v>218</v>
       </c>
@@ -28068,7 +28081,7 @@
         <v/>
       </c>
     </row>
-    <row r="220" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220">
         <v>219</v>
       </c>
@@ -28182,7 +28195,7 @@
         <v/>
       </c>
     </row>
-    <row r="221" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221">
         <v>220</v>
       </c>
@@ -28296,7 +28309,7 @@
         <v>PTG_P1</v>
       </c>
     </row>
-    <row r="222" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A222">
         <v>221</v>
       </c>
@@ -28410,7 +28423,7 @@
         <v>PTG_P1</v>
       </c>
     </row>
-    <row r="223" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223">
         <v>222</v>
       </c>
@@ -28524,7 +28537,7 @@
         <v>PTG_P1</v>
       </c>
     </row>
-    <row r="224" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A224">
         <v>223</v>
       </c>
@@ -28638,7 +28651,7 @@
         <v>PTG_P1</v>
       </c>
     </row>
-    <row r="225" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A225">
         <v>224</v>
       </c>
@@ -28752,7 +28765,7 @@
         <v>PTG_P2</v>
       </c>
     </row>
-    <row r="226" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226">
         <v>225</v>
       </c>
@@ -28866,7 +28879,7 @@
         <v>PTG_P2</v>
       </c>
     </row>
-    <row r="227" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A227">
         <v>226</v>
       </c>
@@ -28980,7 +28993,7 @@
         <v>PTG_P2</v>
       </c>
     </row>
-    <row r="228" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A228">
         <v>227</v>
       </c>
@@ -29094,7 +29107,7 @@
         <v>PTG_P2</v>
       </c>
     </row>
-    <row r="229" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A229">
         <v>228</v>
       </c>
@@ -29208,7 +29221,7 @@
         <v>PTG_P3</v>
       </c>
     </row>
-    <row r="230" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A230">
         <v>229</v>
       </c>
@@ -29322,7 +29335,7 @@
         <v>PTG_P3</v>
       </c>
     </row>
-    <row r="231" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231">
         <v>230</v>
       </c>
@@ -29436,7 +29449,7 @@
         <v>PTG_P3</v>
       </c>
     </row>
-    <row r="232" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A232">
         <v>231</v>
       </c>
@@ -29550,7 +29563,7 @@
         <v>PTG_P3</v>
       </c>
     </row>
-    <row r="233" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A233">
         <v>232</v>
       </c>
@@ -29664,7 +29677,7 @@
         <v>PTG_P4</v>
       </c>
     </row>
-    <row r="234" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A234">
         <v>233</v>
       </c>
@@ -29778,7 +29791,7 @@
         <v>PTG_P4</v>
       </c>
     </row>
-    <row r="235" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235">
         <v>234</v>
       </c>
@@ -29892,7 +29905,7 @@
         <v>PTG_P4</v>
       </c>
     </row>
-    <row r="236" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A236">
         <v>235</v>
       </c>
@@ -30006,7 +30019,7 @@
         <v>PTG_P4</v>
       </c>
     </row>
-    <row r="237" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A237">
         <v>236</v>
       </c>
@@ -30120,7 +30133,7 @@
         <v/>
       </c>
     </row>
-    <row r="238" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A238">
         <v>237</v>
       </c>
@@ -30234,7 +30247,7 @@
         <v/>
       </c>
     </row>
-    <row r="239" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A239">
         <v>238</v>
       </c>
@@ -30348,7 +30361,7 @@
         <v>QMH_4S</v>
       </c>
     </row>
-    <row r="240" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240">
         <v>239</v>
       </c>
@@ -30462,7 +30475,7 @@
         <v/>
       </c>
     </row>
-    <row r="241" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A241">
         <v>240</v>
       </c>
@@ -30576,7 +30589,7 @@
         <v/>
       </c>
     </row>
-    <row r="242" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A242">
         <v>241</v>
       </c>
@@ -30690,7 +30703,7 @@
         <v/>
       </c>
     </row>
-    <row r="243" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A243">
         <v>242</v>
       </c>
@@ -30804,7 +30817,7 @@
         <v/>
       </c>
     </row>
-    <row r="244" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A244">
         <v>243</v>
       </c>
@@ -30918,7 +30931,7 @@
         <v/>
       </c>
     </row>
-    <row r="245" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245">
         <v>244</v>
       </c>
@@ -31032,7 +31045,7 @@
         <v/>
       </c>
     </row>
-    <row r="246" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A246">
         <v>245</v>
       </c>
@@ -31146,7 +31159,7 @@
         <v>QMH_4S</v>
       </c>
     </row>
-    <row r="247" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247">
         <v>246</v>
       </c>
@@ -31260,7 +31273,7 @@
         <v>QMH_4S</v>
       </c>
     </row>
-    <row r="248" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A248">
         <v>247</v>
       </c>
@@ -31374,7 +31387,7 @@
         <v>QMH_4S</v>
       </c>
     </row>
-    <row r="249" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249">
         <v>248</v>
       </c>
@@ -31488,7 +31501,7 @@
         <v>QMH_5a</v>
       </c>
     </row>
-    <row r="250" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A250">
         <v>249</v>
       </c>
@@ -31602,7 +31615,7 @@
         <v>QMH_5a</v>
       </c>
     </row>
-    <row r="251" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251">
         <v>250</v>
       </c>
@@ -31716,7 +31729,7 @@
         <v>QMH_4S</v>
       </c>
     </row>
-    <row r="252" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252">
         <v>251</v>
       </c>
@@ -31830,7 +31843,7 @@
         <v>QMH_4S</v>
       </c>
     </row>
-    <row r="253" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A253">
         <v>252</v>
       </c>
@@ -31944,7 +31957,7 @@
         <v/>
       </c>
     </row>
-    <row r="254" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A254">
         <v>253</v>
       </c>
@@ -32058,7 +32071,7 @@
         <v/>
       </c>
     </row>
-    <row r="255" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A255">
         <v>254</v>
       </c>
@@ -32172,7 +32185,7 @@
         <v/>
       </c>
     </row>
-    <row r="256" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256">
         <v>255</v>
       </c>
@@ -32286,7 +32299,7 @@
         <v/>
       </c>
     </row>
-    <row r="257" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257">
         <v>256</v>
       </c>
@@ -32400,7 +32413,7 @@
         <v/>
       </c>
     </row>
-    <row r="258" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258">
         <v>257</v>
       </c>
@@ -32514,7 +32527,7 @@
         <v/>
       </c>
     </row>
-    <row r="259" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259">
         <v>258</v>
       </c>
@@ -32628,7 +32641,7 @@
         <v/>
       </c>
     </row>
-    <row r="260" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260">
         <v>259</v>
       </c>
@@ -32742,7 +32755,7 @@
         <v/>
       </c>
     </row>
-    <row r="261" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261">
         <v>260</v>
       </c>
@@ -32856,7 +32869,7 @@
         <v/>
       </c>
     </row>
-    <row r="262" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262">
         <v>261</v>
       </c>
@@ -32970,7 +32983,7 @@
         <v/>
       </c>
     </row>
-    <row r="263" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263">
         <v>262</v>
       </c>
@@ -33084,7 +33097,7 @@
         <v/>
       </c>
     </row>
-    <row r="264" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264">
         <v>263</v>
       </c>
@@ -33198,7 +33211,7 @@
         <v/>
       </c>
     </row>
-    <row r="265" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A265">
         <v>264</v>
       </c>
@@ -33312,7 +33325,7 @@
         <v/>
       </c>
     </row>
-    <row r="266" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266">
         <v>265</v>
       </c>
@@ -33426,7 +33439,7 @@
         <v/>
       </c>
     </row>
-    <row r="267" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267">
         <v>266</v>
       </c>
@@ -33540,7 +33553,7 @@
         <v/>
       </c>
     </row>
-    <row r="268" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A268">
         <v>267</v>
       </c>
@@ -33654,7 +33667,7 @@
         <v/>
       </c>
     </row>
-    <row r="269" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269">
         <v>268</v>
       </c>
@@ -33768,7 +33781,7 @@
         <v>TAY_L1</v>
       </c>
     </row>
-    <row r="270" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A270">
         <v>269</v>
       </c>
@@ -33882,7 +33895,7 @@
         <v>TAY_L1</v>
       </c>
     </row>
-    <row r="271" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271">
         <v>270</v>
       </c>
@@ -33996,7 +34009,7 @@
         <v/>
       </c>
     </row>
-    <row r="272" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A272">
         <v>271</v>
       </c>
@@ -34110,7 +34123,7 @@
         <v/>
       </c>
     </row>
-    <row r="273" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A273">
         <v>272</v>
       </c>
@@ -34224,7 +34237,7 @@
         <v/>
       </c>
     </row>
-    <row r="274" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A274">
         <v>273</v>
       </c>
@@ -34338,7 +34351,7 @@
         <v/>
       </c>
     </row>
-    <row r="275" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A275">
         <v>274</v>
       </c>
@@ -34452,7 +34465,7 @@
         <v/>
       </c>
     </row>
-    <row r="276" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A276">
         <v>275</v>
       </c>
@@ -34566,7 +34579,7 @@
         <v/>
       </c>
     </row>
-    <row r="277" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A277">
         <v>276</v>
       </c>
@@ -34680,7 +34693,7 @@
         <v>WES_test_1</v>
       </c>
     </row>
-    <row r="278" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A278">
         <v>277</v>
       </c>
@@ -34794,7 +34807,7 @@
         <v>WES_test_1</v>
       </c>
     </row>
-    <row r="279" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A279">
         <v>278</v>
       </c>
@@ -34908,7 +34921,7 @@
         <v>WES_test_1</v>
       </c>
     </row>
-    <row r="280" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A280">
         <v>279</v>
       </c>
@@ -35022,7 +35035,7 @@
         <v>WES_test_1</v>
       </c>
     </row>
-    <row r="281" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A281">
         <v>280</v>
       </c>
@@ -35136,7 +35149,7 @@
         <v>WES_test_1</v>
       </c>
     </row>
-    <row r="282" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A282">
         <v>281</v>
       </c>
@@ -35250,7 +35263,7 @@
         <v/>
       </c>
     </row>
-    <row r="283" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A283">
         <v>282</v>
       </c>
@@ -35364,7 +35377,7 @@
         <v>ZAN_P1</v>
       </c>
     </row>
-    <row r="284" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A284">
         <v>283</v>
       </c>
@@ -35478,7 +35491,7 @@
         <v>ZAN_P1</v>
       </c>
     </row>
-    <row r="285" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A285">
         <v>284</v>
       </c>
@@ -35592,7 +35605,7 @@
         <v>ZAN_P1</v>
       </c>
     </row>
-    <row r="286" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A286">
         <v>285</v>
       </c>
@@ -35706,7 +35719,7 @@
         <v>ZAN_P1</v>
       </c>
     </row>
-    <row r="287" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A287">
         <v>286</v>
       </c>
@@ -35820,7 +35833,7 @@
         <v/>
       </c>
     </row>
-    <row r="288" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A288">
         <v>287</v>
       </c>
@@ -35934,7 +35947,7 @@
         <v/>
       </c>
     </row>
-    <row r="289" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A289">
         <v>288</v>
       </c>

</xml_diff>